<commit_message>
chore(dashboard): remove codigo orfao do dashboard antigo (ADR 0021)
pages/02_insights.py, pages/03_performance.py e o modulo
src/dashboard/{filters,loaders,comparisons}.py ficaram no repo como
residuo apos a ADR 0021 trocar o entrypoint para dashboard/app.py --
a propria ADR previa remocao incremental, que nao foi cumprida.
Nenhum import ativo restante; so citacoes historicas em docstrings.

Tambem remove DASHBOARD_REFRESH_SECONDS (config/settings.py), config
morta que so servia o auto-refresh do antigo pages/03_performance.py,
e regenera reference/dicionario_de_dados_medallion.xlsx para refletir
os consumidores atuais de cada tabela.

667 testes passam; ruff nao aponta erro novo nos arquivos tocados.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/dicionario_de_dados_medallion.xlsx
+++ b/reference/dicionario_de_dados_medallion.xlsx
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>src/modeling (análise de sentimento, BERTopic); src/dashboard/loaders.py (fallback quando governor_sentiment ainda não existe)</t>
+          <t>src/modeling (análise de sentimento, BERTopic)</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
@@ -1198,7 +1198,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>src/dashboard/filters.py (nome/UF/partido, seletor de governador)</t>
+          <t>dashboard/core/data.py::load_governors_metadata (nome/UF/partido, seletor de governador em todas as telas)</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>src/modeling/growth_history.py (CMGR); pages/03_performance.py (auto-refresh)</t>
+          <t>src/modeling/growth_history.py (CMGR); dashboard/core/data.py::load_engagement_history (comparação vs. média histórica no Resumo, ADR 0025)</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>pages/02_insights.py; src/features/gold/nsm_scorer.py; src/features/gold/topic_priority_scorer.py; scripts/refine_topics.py</t>
+          <t>dashboard/core/data.py::load_sentiment (Resumo, O que produzir, Radar, Discurso x reação); src/features/gold/nsm_scorer.py; src/features/gold/topic_priority_scorer.py; scripts/refine_topics.py</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1768,7 +1768,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>pages/03_performance.py (comparação entre governadores, coeficientes da regressão) -- órfã desde a ADR 0021, sem entrypoint ativo (ver seção 4 do README)</t>
+          <t>Nenhum consumidor de produção hoje -- antigo consumidor (pages/03_performance.py, comparação entre governadores/coeficientes da regressão) era órfão desde a ADR 0021 e foi removido do repositório (cleanup pós-auditoria do dashboard, 2026-10)</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
@@ -1825,7 +1825,7 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>pages/03_performance.py (dispersão previsto vs. real, resíduos) -- órfã desde a ADR 0021, sem entrypoint ativo (ver seção 4 do README)</t>
+          <t>Nenhum consumidor de produção hoje -- antigo consumidor (pages/03_performance.py, dispersão previsto vs. real/resíduos) era órfão desde a ADR 0021 e foi removido do repositório (cleanup pós-auditoria do dashboard, 2026-10)</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Nenhum consumidor de produção hoje -- dashboard/screens/funil.py (Tela 6, ADR 0021) proíbe estruturalmente qualquer referência a esta tabela (ver teste test_funil_module_never_references_ugc_tables); src/dashboard/filters.py tem a função de agregação, mas não é chamada por nenhuma tela atual. Materializada com dado real desde 2026-09-19, mas o funil (Tela 6, issue #114) continua mostrando 'Engage · Criar' como 'em construção' por decisão de design, não por falta de dado.</t>
+          <t>Nenhum consumidor de produção hoje -- dashboard/screens/funil.py (Tela 6, ADR 0021) proíbe estruturalmente qualquer referência a esta tabela (ver teste test_funil_module_never_references_ugc_tables). Materializada com dado real desde 2026-09-19, mas o funil (Tela 6, issue #114) continua mostrando 'Engage · Criar' como 'em construção' por decisão de design, não por falta de dado.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -11812,7 +11812,7 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Dashboard Streamlit (dashboard/app.py + dashboard/screens/*.py, ADR 0021; pages/02-03 remanescentes, órfãs) e notebooks/03-07</t>
+          <t>Dashboard Streamlit (dashboard/app.py + dashboard/screens/*.py, ADR 0021) e notebooks/03-07</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
@@ -11822,7 +11822,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>src/repositories/delta_repository.py + dashboard/core/* + src/dashboard/*</t>
+          <t>src/repositories/delta_repository.py + dashboard/core/*</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(catalogo): documenta governor_scorecard e ICE de pautas no catalogo de dados
Adiciona as tabelas Gold governor_scorecard e content_topic_priority_score
(colunas, origem, regra de calculo e selos de confiabilidade), atualiza
governor_sentiment e governor_discourse_topics (rotulos refinados,
preservacao de legenda/transcricao), a nota de videoPlayCount como
reproducoes (plays), linhagem, glossario e contagem de tabelas. Catalogo
regerado.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/dicionario_de_dados_medallion.xlsx
+++ b/reference/dicionario_de_dados_medallion.xlsx
@@ -17,13 +17,13 @@
     <sheet name="Glossário de Métricas" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tabelas'!$A$1:$K$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tabelas'!$A$1:$K$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Colunas - Bronze'!$A$1:$E$72</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas - Silver'!$A$1:$E$84</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Colunas - Gold'!$A$1:$E$181</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Linhagem'!$A$1:$D$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Colunas - Gold'!$A$1:$E$215</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Linhagem'!$A$1:$D$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Actors Apify'!$A$1:$H$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Glossário de Métricas'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Glossário de Métricas'!$A$1:$E$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -576,7 +576,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Bronze: 4  |  Silver: 6  |  Gold: 13  |  Total: 23</t>
+          <t>Bronze: 4  |  Silver: 6  |  Gold: 17  |  Total: 27</t>
         </is>
       </c>
     </row>
@@ -621,7 +621,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>5. Aba 'Glossário de Métricas' -- fórmula completa de cada métrica derivada (% ENGAJAMENTO, NSM, Score ICE, CMGR, retenção, Y da regressão, cluster_score).</t>
+          <t>5. Aba 'Glossário de Métricas' -- fórmula completa de cada métrica derivada (% ENGAJAMENTO, NSM, Score ICE, CMGR, retenção, Y da regressão, cluster_score, Escore composto, Score ICE por pauta).</t>
         </is>
       </c>
     </row>
@@ -636,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>dashboard/core/data.py::load_sentiment (Resumo, O que produzir, Radar, Discurso x reação); src/features/gold/nsm_scorer.py; src/features/gold/topic_priority_scorer.py; scripts/refine_topics.py</t>
+          <t>dashboard/core/data.py::load_sentiment (Resumo [sub-abas NSM e Funil], O que produzir, Radar, Comparar perfis, Discurso x reação); src/features/gold/nsm_scorer.py; src/features/gold/topic_priority_scorer.py; src/features/gold/content_topic_priority_scorer.py; src/modeling/governor_scorecard.py; scripts/refine_topics.py</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1446,7 +1446,7 @@
       </c>
       <c r="K14" s="3" t="inlineStr">
         <is>
-          <t>`scripts/refine_topics.py` reescreve os rótulos de `Name` via Gemini sobre esta MESMA tabela (não gera nova medição de sentimento) -- ver ADR 0001. NSM e Score ICE filtram só `fonte == 'comentario'`; linhas de legenda/transcrição não entram nessas duas métricas.</t>
+          <t>`scripts/refine_topics.py` reescreve os rótulos de `Name` via Gemini sobre esta MESMA tabela (não gera nova medição de sentimento) -- ver ADR 0001. A escrita do refino (issue #186) é overwrite SÓ das linhas `fonte == 'comentario'`: as linhas de legenda e transcrição gravadas pela modelagem determinística são PRESERVADAS (antes do #186 o refino apagava essas linhas). NSM, Score ICE (comentário e pauta) e Escore composto (dimensão Qualidade) filtram só `fonte == 'comentario'`; linhas de legenda/transcrição não entram nessas métricas.</t>
         </is>
       </c>
     </row>
@@ -1540,7 +1540,7 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>dashboard/screens/{resumo,produzir,discurso_reacao,funil}.py (ADR 0021)</t>
+          <t>dashboard/screens/{produzir,discurso_reacao}.py (ADR 0021); src/features/gold/content_topic_priority_scorer.py (pauta de cada reel pela legenda)</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
@@ -1550,17 +1550,17 @@
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>ADR 0020 Ficha 4 / issue #89</t>
+          <t>ADR 0020 Ficha 4 / issue #89; issue #186 (refino Gemini do discurso)</t>
         </is>
       </c>
       <c r="J16" s="3" t="inlineStr">
         <is>
-          <t>Tópicos do que a ASSESSORIA publica (legenda de post/reel + transcrição de fala) -- BERTopic próprio, não misturado ao de comentário.</t>
+          <t>Tópicos do que a ASSESSORIA publica (legenda de post/reel + transcrição de fala) -- BERTopic próprio, não misturado ao de comentário. Cada tópico de legenda é uma PAUTA (assunto do conteúdo) na fila de "O que produzir".</t>
         </is>
       </c>
       <c r="K16" s="3" t="inlineStr">
         <is>
-          <t>Conceitualmente distinta de governor_sentiment: fala da assessoria (aqui) vs. reação do público (lá). Nunca comparar os `Topic`/`Name` das duas tabelas como se fossem o mesmo espaço de tópicos.</t>
+          <t>Conceitualmente distinta de governor_sentiment: fala da assessoria (aqui) vs. reação do público (lá). Nunca comparar os `Topic`/`Name` das duas tabelas como se fossem o mesmo espaço de tópicos. RÓTULOS REFINADOS (issue #186): `Name` sai do modelo determinístico como `&lt;id&gt;_kw1_kw2...` (ou `1____` quando o tópico não tem palavra alguma); o refino manual (`scripts/refine_topics.py --target all|discourse`, fora do pipeline automático) troca por `&lt;id&gt;_&lt;rótulo legível&gt;_&lt;kw...&gt;`. O tópico de ruído (`-1`) nunca é refinado e mantém o `Name` que já tinha; o tópico degenerado (sem palavra alguma) recebe o rótulo fixo "sem assunto definido" em vez de um nome inventado. O refino escreve nesta MESMA tabela (overwrite) e recalcula `content_topic_priority_score`. Enquanto o refino real não for rodado, os rótulos são os provisórios do estágio determinístico.</t>
         </is>
       </c>
     </row>
@@ -1597,7 +1597,7 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>dashboard/screens/{resumo,produzir,funil}.py (ADR 0021)</t>
+          <t>dashboard/screens/{produzir,comparar_clusters,resumo_funil}.py (ADR 0021; análise de clusters de reels em Comparar perfis, issue #189)</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
@@ -1882,7 +1882,7 @@
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>dashboard/screens/{resumo,produzir,radar}.py (priorização do que produzir a seguir, ADR 0021)</t>
+          <t>dashboard/screens/radar.py (tópicos de comentário em alerta). Desde a issue #191 a fila de "O que produzir" lê `content_topic_priority_score` (pautas), não esta tabela</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
@@ -1897,7 +1897,7 @@
       </c>
       <c r="J22" s="3" t="inlineStr">
         <is>
-          <t>Score ICE (Impacto x Confiança x Facilidade) de priorização de tópicos de comentário -- responde 'sobre o que o governador deveria produzir a seguir'.</t>
+          <t>Score ICE (Impacto x Confiança x Facilidade) de priorização de tópicos de COMENTÁRIO (grupos de comentários) -- não confundir com `content_topic_priority_score`, o ICE por PAUTA (assunto do conteúdo) que alimenta a fila de "O que produzir".</t>
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>dashboard/screens/resumo.py (Tela 1, ADR 0021)</t>
+          <t>dashboard/screens/resumo_nsm.py (Resumo, sub-aba NSM, ADR 0031 / issue #187)</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
@@ -1996,7 +1996,7 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>dashboard/core/data.py::load_nsm_history() -&gt; dashboard/screens/resumo.py (Tela 1, delta "vs. média histórica" do KPI Engajamento qualificado)</t>
+          <t>dashboard/core/data.py::load_nsm_history() -&gt; dashboard/screens/resumo_nsm.py (Resumo, sub-aba NSM, delta "vs. média histórica" do KPI Engajamento qualificado)</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
@@ -2053,7 +2053,7 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>Nenhum consumidor de produção hoje -- dashboard/screens/funil.py (Tela 6, ADR 0021) proíbe estruturalmente qualquer referência a esta tabela (ver teste test_funil_module_never_references_ugc_tables). Materializada com dado real desde 2026-09-19, mas o funil (Tela 6, issue #114) continua mostrando 'Engage · Criar' como 'em construção' por decisão de design, não por falta de dado.</t>
+          <t>Nenhum consumidor de produção hoje -- dashboard/screens/resumo_funil.py (sub-aba Funil do Resumo, ADR 0031; antiga Tela 6) proíbe estruturalmente qualquer referência a esta tabela (ver teste test_funil_module_never_references_ugc_tables). Materializada com dado real desde 2026-09-19, mas o funil (issue #114) continua mostrando 'Engage · Criar' como 'em construção' por decisão de design, não por falta de dado.</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>Nenhuma tela do dashboard atual (ADR 0021) consome esta tabela -- dashboard/core/data.py::load_growth_metrics() existe, mas não é chamada por nenhuma das 6 telas</t>
+          <t>dashboard/screens/resumo_nsm.py (KPIs de crescimento CMGR e retenção, Resumo sub-aba NSM) via dashboard/core/data.py::load_growth_metrics()</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
@@ -2134,8 +2134,122 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>data/gold/governor_scorecard</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Uma linha por governador (um perfil por `inputUrl` normalizado) -- snapshot recalculável a partir da Silver/Gold atual, sempre overwrite.</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>src/modeling/governor_scorecard.py (GovernorScorecardScorer), via src/modeling/orchestration.py::run_deterministic_modeling (pipeline.py --run-modeling / scripts/run_modeling.py) ou, isoladamente, scripts/run_governor_scorecard.py</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>dashboard/screens/resumo_scorecard.py (Resumo, sub-aba Scorecard) via dashboard/core/data.py::load_governor_scorecard() -- o dashboard só lê, nada é recalculado</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>Produção -- com selo de confiabilidade: dimensão Consistência pendente nos 26 governadores no dado de 2026-10-04 (ver notas)</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>ADR 0030 / issue #184 (spec #182)</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Escore composto (0 a 100) dos governadores: soma ponderada de cinco dimensões normalizadas min-máx entre os perfis (Alcance, Ativação, Qualidade, Profundidade, Consistência), seguindo a lógica de indicadores compostos do OECD Handbook (indicador bruto -&gt; normalização -&gt; ponderação -&gt; agregação). Relativo ao grupo: mede posição entre pares, não desempenho absoluto.</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>SELOS DE CONFIABILIDADE. (1) Alcance é medido em REPRODUÇÕES (plays: `videoPlayCount` dos reels), nunca em "visualizações únicas"; posts de feed não têm plays, então só reels entram em Alcance e Profundidade. (2) Consistência mede a TENDÊNCIA do engajamento médio por post por mês de publicação (CMGR de engajamento), NÃO crescimento de audiência -- o CMGR de audiência (seguidores entre coletas, `governor_growth_metrics.cmgr`) continua pendente e fora do escore. (3) Consistência exige &gt;= 4 meses completos com &gt;= 3 posts maduros (&gt;= 7 dias de vida); no dado de 2026-10-04 a Silver só tem ~226 posts de ago/set-2026 e NENHUM dos 26 governadores atinge isso, então `consistencia_pendente = True` e `consistencia`/`consistencia_norm` são nulas em todos: o escore usa as 4 dimensões restantes com peso 0,25 cada (com as 5, 0,20 cada) e `n_dimensoes = 4`. Isso muda sozinho conforme a Silver acumular histórico. (4) Perfil com menos de 4 dimensões disponíveis fica com `escore` e `ranking` nulos. (5) São 26 governadores (a Silver filtra governadores removidos de governadores.xlsx), não 27. Amplitude zero numa dimensão (todos iguais) normaliza para 50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Gold</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>data/gold/content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Uma linha por PAUTA (tópico de discurso da legenda do reel) -- ranking global, todos os perfis combinados, não por governador.</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>overwrite</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>src/features/gold/content_topic_priority_scorer.py (ContentTopicPriorityScorer), via src/modeling/orchestration.py::run_deterministic_modeling (provisório, rótulos brutos) e refine_discourse_topics_with_gemini (recalculado com os rótulos refinados)</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>dashboard/screens/produzir.py (fila de pautas de "O que produzir") via dashboard/core/data.py::load_content_topic_priority()</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Produção -- com selo de confiabilidade: rótulos de pauta ainda provisórios até o refino manual via Gemini ser rodado de verdade (ver notas)</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>ADR 0020 Ficha 6 (fórmula); ADR 0028; issue #190 / #191 (spec #182)</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Score ICE (Impacto x Confiança x Facilidade) por PAUTA: sobre qual assunto de conteúdo o público reagiu bem. Pauta = tópico de discurso da LEGENDA do reel; os comentários são ligados à pauta pelo reel (`id_reel`).</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Cada reel pertence a uma única pauta (a da legenda; `governor_discourse_topics` tem reels duplicados, deduplicados por `id_reel`); comentários de reels sem pauta de legenda ficam de fora; o tópico de ruído (-1) não é pauta; a transcrição não define pauta (exige plano pago do coletor). `alcance_pauta` é PROXY por engajamento (soma de likesCount + repliesCount dos comentários), nunca "visualizações". `facilidade` fixa em 1,0 (v1, sem dado de custo de produção). O selo de prioridade do dashboard (Alta/Média/Cuidado) vem dos tercis de `score` sobre o ranking global de pautas; o score bruto nunca é exibido. SELO DE CONFIABILIDADE: o refino real dos rótulos via Gemini ainda não foi rodado -- até lá `Name` traz os rótulos provisórios do BERTopic (palavras-chave) e o tópico sem palavra alguma aparece como "sem assunto definido". O ICE é recalculado quando o refino do discurso roda (`scripts/refine_topics.py --target all|discourse`).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K26"/>
+  <autoFilter ref="A1:K28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2962,7 +3076,7 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3427,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -3880,7 +3994,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4988,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -5171,7 +5285,7 @@
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -6278,7 +6392,7 @@
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -6402,7 +6516,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E181"/>
+  <dimension ref="A1:E215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -10755,7 +10869,7 @@
       </c>
       <c r="E161" s="3" t="inlineStr">
         <is>
-          <t>Número de plays do vídeo (Reels/vídeo de feed).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -11299,8 +11413,926 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>inputUrl</t>
+        </is>
+      </c>
+      <c r="C182" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D182" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E182" s="3" t="inlineStr">
+        <is>
+          <t>URL do perfil do governador (chave de junção; normalizada em minúsculas, sem espaços e sem barra final para cruzar Silver e Gold).</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>username</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D183" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E183" s="3" t="inlineStr">
+        <is>
+          <t>Username do perfil (de governor_engagement); pode ser nulo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>alcance</t>
+        </is>
+      </c>
+      <c r="C184" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D184" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E184" s="3" t="inlineStr">
+        <is>
+          <t>Dimensão Alcance bruta: média de videoPlayCount (REPRODUÇÕES / plays, nunca "visualizações únicas") dos reels do perfil. Posts de feed não têm plays e não entram. Nulo sem reels com plays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>ativacao</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D185" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E185" s="3" t="inlineStr">
+        <is>
+          <t>Dimensão Ativação bruta: média de likesCount dos reels / followersCount do perfil. Nulo sem reels ou sem seguidores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>qualidade</t>
+        </is>
+      </c>
+      <c r="C186" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D186" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E186" s="3" t="inlineStr">
+        <is>
+          <t>Dimensão Qualidade bruta: comentários positivos / comentários totais do perfil (só governor_sentiment com fonte == 'comentario'). Nulo sem comentários.</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>profundidade</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D187" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E187" s="3" t="inlineStr">
+        <is>
+          <t>Dimensão Profundidade bruta: média de commentsCount / média de videoPlayCount, ambas sobre os reels com plays (mesma base do Alcance). Nulo sem reels com plays.</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>consistencia</t>
+        </is>
+      </c>
+      <c r="C188" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D188" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E188" s="3" t="inlineStr">
+        <is>
+          <t>Dimensão Consistência bruta: CMGR de engajamento por data de publicação = exp(inclinação) - 1 da regressão log-linear sobre o engajamento médio por post (curtidas + comentários) de cada mês de publicação. Janela de até 12 meses completos (mês corrente excluído), mês válido com &gt;= 3 posts, posts com &lt; 7 dias de vida excluídos. Nula (pendente) com &lt; 4 meses válidos. NÃO é crescimento de audiência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>alcance_norm</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D189" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E189" s="3" t="inlineStr">
+        <is>
+          <t>alcance normalizado min-máx 0-100 entre os perfis com a dimensão (100 = maior). Amplitude zero -&gt; 50. Nulo quando a dimensão bruta é nula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>ativacao_norm</t>
+        </is>
+      </c>
+      <c r="C190" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D190" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E190" s="3" t="inlineStr">
+        <is>
+          <t>ativacao normalizada min-máx 0-100 entre os perfis (mesma regra de alcance_norm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>qualidade_norm</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D191" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E191" s="3" t="inlineStr">
+        <is>
+          <t>qualidade normalizada min-máx 0-100 entre os perfis (mesma regra de alcance_norm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>profundidade_norm</t>
+        </is>
+      </c>
+      <c r="C192" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D192" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E192" s="3" t="inlineStr">
+        <is>
+          <t>profundidade normalizada min-máx 0-100 entre os perfis (mesma regra de alcance_norm).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>consistencia_norm</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D193" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E193" s="3" t="inlineStr">
+        <is>
+          <t>consistencia normalizada min-máx 0-100 entre os perfis com a dimensão. Nula quando Consistência está pendente (hoje, todos os 26 governadores).</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>consistencia_pendente</t>
+        </is>
+      </c>
+      <c r="C194" s="3" t="inlineStr">
+        <is>
+          <t>bool</t>
+        </is>
+      </c>
+      <c r="D194" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E194" s="3" t="inlineStr">
+        <is>
+          <t>True quando a Consistência não pôde ser calculada (&lt; 4 meses válidos). Selo de confiabilidade: o escore daquele perfil usa só as outras dimensões, com os pesos renormalizados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>consistencia_n_meses</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D195" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E195" s="3" t="inlineStr">
+        <is>
+          <t>Número de meses de publicação válidos (&gt;= 3 posts maduros, dentro da janela) que entraram, ou entrariam, no cálculo da Consistência.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>n_dimensoes</t>
+        </is>
+      </c>
+      <c r="C196" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D196" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E196" s="3" t="inlineStr">
+        <is>
+          <t>Quantas das 5 dimensões normalizadas entraram no escore deste perfil (5, ou 4 com Consistência pendente). Perfil com &lt; 4 fica sem escore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>escore</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D197" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E197" s="3" t="inlineStr">
+        <is>
+          <t>Escore composto 0-100: média simples das dimensões normalizadas disponíveis (soma ponderada com pesos iguais: 0,20 com 5 dimensões, 0,25 com 4). Nulo com &lt; 4 dimensões. Relativo ao grupo de perfis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>ranking</t>
+        </is>
+      </c>
+      <c r="C198" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D198" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E198" s="3" t="inlineStr">
+        <is>
+          <t>Posição do perfil pelo escore (1 = maior; desempate por inputUrl). Nulo quando o perfil não tem escore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>_run_id</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D199" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E199" s="3" t="inlineStr">
+        <is>
+          <t>Identificador da execução do pipeline que gravou a linha (src/run_id.py) -- rastreia de qual chamada de pipeline.py/scripts/*.py a linha se origina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>governor_scorecard</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>_generated_at</t>
+        </is>
+      </c>
+      <c r="C200" s="3" t="inlineStr">
+        <is>
+          <t>timestamp[us, tz=UTC]</t>
+        </is>
+      </c>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E200" s="3" t="inlineStr">
+        <is>
+          <t>Timestamp UTC de quando a linha foi calculada/gravada na Gold -- distinto de _ingested_at (que é do dado bruto na Bronze).</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D201" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E201" s="3" t="inlineStr">
+        <is>
+          <t>Id numérico do tópico de DISCURSO (BERTopic de legendas) que define a pauta -- espaço de ids distinto do tópico de comentário. O ruído (-1) nunca é pauta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C202" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D202" s="3" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="E202" s="3" t="inlineStr">
+        <is>
+          <t>Rótulo da pauta: tópico de discurso sem o prefixo de id; rótulo refinado via Gemini quando o refino do discurso rodou, palavras-chave separadas por vírgula quando provisório, ou "sem assunto definido" quando o tópico é degenerado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>n_reels</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D203" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E203" s="3" t="inlineStr">
+        <is>
+          <t>Número de reels distintos cuja legenda pertence à pauta e que receberam ao menos um comentário.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>n_comentarios</t>
+        </is>
+      </c>
+      <c r="C204" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D204" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E204" s="3" t="inlineStr">
+        <is>
+          <t>Número de comentários (fonte == 'comentario') dos reels da pauta -- cada reel conta numa única pauta, então os totais somam o total real de comentários com pauta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>n_comentarios_positivos</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D205" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E205" s="3" t="inlineStr">
+        <is>
+          <t>Comentários da pauta com sentiment_label == 'positive'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>n_comentarios_negativos</t>
+        </is>
+      </c>
+      <c r="C206" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D206" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E206" s="3" t="inlineStr">
+        <is>
+          <t>Comentários da pauta com sentiment_label == 'negative'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>proporcao_sentimento_positivo</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D207" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E207" s="3" t="inlineStr">
+        <is>
+          <t>n_comentarios_positivos / n_comentarios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>alcance_pauta</t>
+        </is>
+      </c>
+      <c r="C208" s="3" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="D208" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E208" s="3" t="inlineStr">
+        <is>
+          <t>Soma de (likesCount + repliesCount) dos comentários da pauta -- PROXY por engajamento, não alcance nem visualizações reais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>alcance_normalizado</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D209" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E209" s="3" t="inlineStr">
+        <is>
+          <t>alcance_pauta / (alcance_pauta + 1) -- satura suavemente em [0,1), estável entre execuções.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>confianca</t>
+        </is>
+      </c>
+      <c r="C210" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D210" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E210" s="3" t="inlineStr">
+        <is>
+          <t>Média de sentiment_score (confiança do classificador, não polaridade) dos comentários da pauta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>impacto</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D211" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E211" s="3" t="inlineStr">
+        <is>
+          <t>alcance_normalizado x proporcao_sentimento_positivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>facilidade</t>
+        </is>
+      </c>
+      <c r="C212" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D212" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E212" s="3" t="inlineStr">
+        <is>
+          <t>Fixa em 1,0 (v1) -- sem dado de custo de produção real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>score</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>double</t>
+        </is>
+      </c>
+      <c r="D213" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E213" s="3" t="inlineStr">
+        <is>
+          <t>Impacto x Confiança x Facilidade -- base do selo de prioridade (Alta/Média/Cuidado por tercis do ranking global de pautas) na fila de "O que produzir".</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>_run_id</t>
+        </is>
+      </c>
+      <c r="C214" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D214" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E214" s="3" t="inlineStr">
+        <is>
+          <t>Identificador da execução do pipeline que gravou a linha (src/run_id.py) -- rastreia de qual chamada de pipeline.py/scripts/*.py a linha se origina.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="3" t="inlineStr">
+        <is>
+          <t>content_topic_priority_score</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>_generated_at</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>timestamp[us, tz=UTC]</t>
+        </is>
+      </c>
+      <c r="D215" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E215" s="3" t="inlineStr">
+        <is>
+          <t>Timestamp UTC de quando a linha foi calculada/gravada na Gold -- distinto de _ingested_at (que é do dado bruto na Bronze).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E181"/>
+  <autoFilter ref="A1:E215"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11311,7 +12343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -11763,71 +12795,137 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Gold: governor_engagement_history + governor_sentiment_history</t>
+          <t>Gold: governor_sentiment (fonte='comentario') + governor_discourse_topics (fonte='legenda')</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Gold: governor_growth_metrics</t>
+          <t>Gold: content_topic_priority_score</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>CMGR sobre followersCount mensal + retenção sobre share mensal de sentimento positivo; marca ilustrativo/confiavel conforme volume de histórico.</t>
+          <t>Score ICE por pauta: comentários ligados à pauta do reel (legenda) via id_reel; Impacto(alcance_normalizado x %positivo) x Confiança(sentiment_score médio) x Facilidade(fixa=1,0), agregado por Topic de discurso. Calculado de forma provisória no estágio determinístico e recalculado após o refino Gemini do discurso.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>src/modeling/growth_history.py + scripts/run_growth_metrics.py</t>
+          <t>src/features/gold/content_topic_priority_scorer.py (orchestration.py::run_deterministic_modeling e refine_discourse_topics_with_gemini)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Apify (apify/instagram-tagged-scraper -- ver aba Actors Apify)</t>
+          <t>Gold: governor_discourse_topics</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Bronze/Silver/Gold: ugc_mentions / governor_ugc_mentions</t>
+          <t>governor_discourse_topics (rótulos refinados)</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Coleta -&gt; landing zone -&gt; Bronze -&gt; Silver (dedup id/shortCode, normalização de handle, resolução de governor_username via mentions+taggedUsers) -&gt; Gold (is_organic a partir de paidPartnership), tudo sob o mesmo run_id -- mesmo padrão de scripts/run_apify_backfill.py. Schema corrigido contra o piloto real (scripts/run_apify_mentions_pilot.py, 2026-09-19, data/pilot/*.json, fora do Delta Lake). Writer de produção rodou contra a Apify de produção pela 1a vez em 2026-09-19 (achado no PR #140, que corrigiu um FutureWarning de pandas revelado por esse dado real).</t>
+          <t>Refinamento manual dos rótulos de tópico de discurso (Name) via Gemini; ruído (-1) mantido, tópico degenerado vira "sem assunto definido". Reescreve a mesma tabela e recalcula content_topic_priority_score.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>scripts/run_ugc_mentions.py + src/data_extract/bronze_writer.py + src/features/silver/ugc_mention_cleaner.py + src/features/gold/ugc_mentions_aggregator.py</t>
+          <t>scripts/refine_topics.py (--target all|discourse) + src/modeling/orchestration.py::refine_discourse_topics_with_gemini</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>Gold: governor_engagement (seguidores) + Silver: reels_clean + posts_clean + Gold: governor_sentiment (fonte='comentario')</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Gold: governor_scorecard</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Escore composto: 5 dimensões por governador (Alcance, Ativação, Qualidade, Profundidade, Consistência), normalização min-máx 0-100 entre os perfis, média simples das dimensões disponíveis (pesos iguais renormalizados), ranking. Consistência = CMGR de engajamento por data de publicação (pendente sem &gt;= 4 meses válidos).</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>src/modeling/governor_scorecard.py (orchestration.py::run_deterministic_modeling ou scripts/run_governor_scorecard.py)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Gold: governor_engagement_history + governor_sentiment_history</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Gold: governor_growth_metrics</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>CMGR sobre followersCount mensal + retenção sobre share mensal de sentimento positivo; marca ilustrativo/confiavel conforme volume de histórico.</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>src/modeling/growth_history.py + scripts/run_growth_metrics.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Apify (apify/instagram-tagged-scraper -- ver aba Actors Apify)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Bronze/Silver/Gold: ugc_mentions / governor_ugc_mentions</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Coleta -&gt; landing zone -&gt; Bronze -&gt; Silver (dedup id/shortCode, normalização de handle, resolução de governor_username via mentions+taggedUsers) -&gt; Gold (is_organic a partir de paidPartnership), tudo sob o mesmo run_id -- mesmo padrão de scripts/run_apify_backfill.py. Schema corrigido contra o piloto real (scripts/run_apify_mentions_pilot.py, 2026-09-19, data/pilot/*.json, fora do Delta Lake). Writer de produção rodou contra a Apify de produção pela 1a vez em 2026-09-19 (achado no PR #140, que corrigiu um FutureWarning de pandas revelado por esse dado real).</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>scripts/run_ugc_mentions.py + src/data_extract/bronze_writer.py + src/features/silver/ugc_mention_cleaner.py + src/features/gold/ugc_mentions_aggregator.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
           <t>Gold (todas as tabelas acima)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B26" s="3" t="inlineStr">
         <is>
           <t>Dashboard Streamlit (dashboard/app.py + dashboard/screens/*.py, ADR 0021) e notebooks/03-07</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Leitura read-only via src/repositories/delta_repository.py (DeltaRepository) -- nunca escreve, save() levanta NotImplementedError deliberadamente.</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D26" s="3" t="inlineStr">
         <is>
           <t>src/repositories/delta_repository.py + dashboard/core/*</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D23"/>
+  <autoFilter ref="A1:D26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -12073,7 +13171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -12275,113 +13373,194 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>CMGR (governor_growth_metrics.cmgr)</t>
+          <t>Score ICE por pauta (content_topic_priority_score.score)</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>governor_growth_metrics</t>
+          <t>content_topic_priority_score</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>(valor_final / valor_inicial) ** (1 / n_meses) - 1, sobre followersCount mensal</t>
+          <t>Impacto x Confiança x Facilidade, onde Impacto = alcance_normalizado x %positivo, alcance_normalizado = alcance_pauta/(alcance_pauta+1), alcance_pauta = soma de (likes+replies) dos comentários dos reels da pauta</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Crescimento mensal composto de seguidores -- ADR 0020 Ficha 7.</t>
+          <t>Ranking de priorização de PAUTAS (assunto da legenda) para a fila de "O que produzir" -- sobre qual assunto de conteúdo o público reagiu bem. Spec #182 / issue #190.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>cmgr_confiavel=False com menos de 6 execuções mensais acumuladas -- resultado atual (2026-09) é ILUSTRATIVO, valida a fórmula, não sustenta conclusão real no TCC.</t>
+          <t>Facilidade fixa em 1,0; alcance_pauta é proxy por engajamento, não views reais; rótulos de pauta provisórios até o refino Gemini real ser rodado; reel sem pauta de legenda fica de fora.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Retenção (governor_growth_metrics.retencao)</t>
+          <t>Escore composto (governor_scorecard.escore)</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>governor_growth_metrics</t>
+          <t>governor_scorecard</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Média (capada em 1.0) de valor_t/valor_(t-1) do share mensal de sentimento positivo entre meses consecutivos</t>
+          <t>Média simples das dimensões normalizadas (min-máx 0-100 entre os perfis) disponíveis: Alcance, Ativação, Qualidade, Profundidade, Consistência. Pesos iguais: 0,20 com 5 dimensões, 0,25 com 4 (Consistência pendente).</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Quanto do sentimento positivo do mês anterior foi mantido -- mede retenção, não crescimento (CMGR cobre magnitude).</t>
+          <t>Posição relativa do governador entre os pares, decomponível por dimensão -- ADR 0030 / issue #184.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Mesma ressalva de confiabilidade do CMGR (min. 6 períodos).</t>
+          <t>Relativo ao grupo (26 perfis hoje), não desempenho absoluto. Alcance = reproduções (plays) só de reels. Consistência pendente nos 26 perfis no dado de 2026-10-04 (histórico de publicação curto) -- hoje o escore é de 4 dimensões. Perfil com &lt; 4 dimensões não tem escore.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Y da regressão de performance-por-post</t>
+          <t>CMGR de engajamento (governor_scorecard.consistencia)</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>post_performance_predictions (y_real/y_previsto/residuo)</t>
+          <t>governor_scorecard</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>(likesCount + commentsCount × _WC_COMENTARIO) / followersCount, por POST (não por perfil)</t>
+          <t>exp(inclinação da regressão log-linear do engajamento médio por post por mês de publicação) - 1; janela de até 12 meses completos, mês com &gt;= 3 posts, posts com &gt;= 7 dias de vida, &gt;= 4 meses válidos</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Mesma lógica ponderada de % ENGAJAMENTO, mas na granularidade de post individual -- variável explicada pela regressão Lasso (ADR 0019 parte C).</t>
+          <t>Tendência mensal composta do engajamento dos posts por data de publicação (ADR 0030). Distinto do CMGR de audiência (seguidores entre coletas).</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Preditores derivados das mesmas colunas brutas de Y são bloqueados por checagem de circularidade (CircularityError) antes do treino.</t>
+          <t>Não mede crescimento de audiência. Nula quando o histórico de publicação é curto (hoje, todos os perfis).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
+          <t>CMGR (governor_growth_metrics.cmgr)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>governor_growth_metrics</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>(valor_final / valor_inicial) ** (1 / n_meses) - 1, sobre followersCount mensal</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Crescimento mensal composto de seguidores -- ADR 0020 Ficha 7.</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>cmgr_confiavel=False com menos de 6 execuções mensais acumuladas -- resultado atual (2026-09) é ILUSTRATIVO, valida a fórmula, não sustenta conclusão real no TCC.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Retenção (governor_growth_metrics.retencao)</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>governor_growth_metrics</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Média (capada em 1.0) de valor_t/valor_(t-1) do share mensal de sentimento positivo entre meses consecutivos</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Quanto do sentimento positivo do mês anterior foi mantido -- mede retenção, não crescimento (CMGR cobre magnitude).</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Mesma ressalva de confiabilidade do CMGR (min. 6 períodos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Y da regressão de performance-por-post</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>post_performance_predictions (y_real/y_previsto/residuo)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>(likesCount + commentsCount × _WC_COMENTARIO) / followersCount, por POST (não por perfil)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Mesma lógica ponderada de % ENGAJAMENTO, mas na granularidade de post individual -- variável explicada pela regressão Lasso (ADR 0019 parte C).</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Preditores derivados das mesmas colunas brutas de Y são bloqueados por checagem de circularidade (CircularityError) antes do treino.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>cluster_score (governor_clusters_reels / governor_clusters_posts / governor_profile_clusters_engagement)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>governor_clusters_reels / governor_clusters_posts / governor_profile_clusters_engagement</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Silhouette + Calinski-Harabasz normalizado (tanh(chi/10000)) + Davies-Bouldin invertido (tanh(1/dbi)), combinado</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>Score CVI (Cluster Validity Index) combinado usado pelo AutoClusterHPO para eleger o algoritmo/hiperparâmetros de clusterização.</t>
         </is>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>Pontos de ruído do DBSCAN (cluster_label=-1) são filtrados ANTES do cálculo do CVI, para não distorcer a comparação entre algoritmos.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E11"/>
+  <autoFilter ref="A1:E14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: renumera ADR do pipeline para 0034 e corrige achados do code review
A ADR do pipeline como ponto unico colidia com a 0033 do comparativo vs
mediana; vira 0034, com citacoes atualizadas (README, CONTEXT, catalogo
regenerado) e nota de superseded parcial na ADR 0020. Tambem: anotacao de
retorno de extract_and_land coerente com ugc_error, relatorio de tabelas
sempre mostra a pasta de logs e exemplo do README alinhado a saida real.

Refs #224

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/dicionario_de_dados_medallion.xlsx
+++ b/reference/dicionario_de_dados_medallion.xlsx
@@ -1208,7 +1208,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>ADR 0033</t>
+          <t>ADR 0034</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
@@ -8253,7 +8253,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Publicação em que o comentário foi feito: 'reel' (comments_clean) ou 'post' (post_comments_clean) -- só nas linhas fonte == 'comentario'; nula em legenda/transcrição (issue #212, ADR 0033). Não confundir com `fonte`.</t>
+          <t>Publicação em que o comentário foi feito: 'reel' (comments_clean) ou 'post' (post_comments_clean) -- só nas linhas fonte == 'comentario'; nula em legenda/transcrição (issue #212, ADR 0034). Não confundir com `fonte`.</t>
         </is>
       </c>
     </row>
@@ -8685,7 +8685,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Publicação em que o comentário foi feito: 'reel' (comments_clean) ou 'post' (post_comments_clean) -- só nas linhas fonte == 'comentario'; nula em legenda/transcrição (issue #212, ADR 0033). Não confundir com `fonte`.</t>
+          <t>Publicação em que o comentário foi feito: 'reel' (comments_clean) ou 'post' (post_comments_clean) -- só nas linhas fonte == 'comentario'; nula em legenda/transcrição (issue #212, ADR 0034). Não confundir com `fonte`.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(dicionario): precos reais dos actors Apify e IDs tecnicos
Aba "Actors Apify" ganha a coluna "Preco por resultado" com os precos por
plano reverificados em 2026-10-13 na API publica da Apify, os IDs tecnicos dos
tres actors resolvidos por slug e a correcao do "~US$ 1,00/1.000" (posts e
reels) e "US$ 1,50/1.000" (tagged), que estavam desatualizados.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reference/dicionario_de_dados_medallion.xlsx
+++ b/reference/dicionario_de_dados_medallion.xlsx
@@ -18,11 +18,11 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Tabelas'!$A$1:$K$28</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Colunas - Bronze'!$A$1:$E$77</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas - Silver'!$A$1:$E$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Colunas - Bronze'!$A$1:$E$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Colunas - Silver'!$A$1:$E$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Colunas - Gold'!$A$1:$E$206</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Linhagem'!$A$1:$D$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Actors Apify'!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Actors Apify'!$A$1:$I$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Glossário de Métricas'!$A$1:$E$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2267,7 +2267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -3176,12 +3176,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>latestComments</t>
+          <t>isPinned</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Lista bruta (JSON) dos comentários mais recentes do reel ou post, retornada pelo Apify -- fonte de comments_clean (reels) e de post_comments_clean (posts de feed, issue #212).</t>
+          <t>Se o reel está fixado no perfil.</t>
         </is>
       </c>
     </row>
@@ -3203,22 +3203,22 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>latestComments</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Lista bruta (JSON) dos comentários mais recentes do reel ou post, retornada pelo Apify -- fonte de comments_clean (reels) e de post_comments_clean (posts de feed, issue #212).</t>
         </is>
       </c>
     </row>
@@ -3230,12 +3230,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
@@ -3257,7 +3257,7 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>_source</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
@@ -3272,7 +3272,7 @@
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
@@ -3284,7 +3284,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>_raw</t>
+          <t>_source</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -3299,19 +3299,19 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Bronze fiel (ADR 0039): o item COMPLETO retornado pela Apify, serializado como JSON string (ensure_ascii=False), inclusive campos que as colunas tipadas não modelam. Fonte para reprocessar a Silver sem nova extração; parsing e validação ficam na Silver. Substitui a antiga landing zone.</t>
+          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>instagram_reels</t>
+          <t>instagram_posts</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>_raw</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -3321,12 +3321,12 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
+          <t>Bronze fiel (ADR 0039): o item COMPLETO retornado pela Apify, serializado como JSON string (ensure_ascii=False), inclusive campos que as colunas tipadas não modelam. Fonte para reprocessar a Silver sem nova extração; parsing e validação ficam na Silver. Substitui a antiga landing zone.</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>ownerId</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Id do perfil (Bronze/Instagram) que publicou o post/reel.</t>
+          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>ownerUsername</t>
+          <t>ownerId</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Username do perfil que publicou o post/reel/comentário.</t>
+          <t>Id do perfil (Bronze/Instagram) que publicou o post/reel.</t>
         </is>
       </c>
     </row>
@@ -3392,7 +3392,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>inputUrl</t>
+          <t>ownerUsername</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
+          <t>Username do perfil que publicou o post/reel/comentário.</t>
         </is>
       </c>
     </row>
@@ -3419,12 +3419,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>commentsCount</t>
+          <t>inputUrl</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -3434,7 +3434,7 @@
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Número de comentários.</t>
+          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
         </is>
       </c>
     </row>
@@ -3446,7 +3446,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>commentsCount</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -3461,7 +3461,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Número de comentários.</t>
         </is>
       </c>
     </row>
@@ -3473,7 +3473,7 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>videoViewCount</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -3488,7 +3488,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Número de views do vídeo (métrica bruta do Apify, distinta de videoPlayCount).</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>videoPlayCount</t>
+          <t>videoViewCount</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
+          <t>Número de views do vídeo (métrica bruta do Apify, distinta de videoPlayCount).</t>
         </is>
       </c>
     </row>
@@ -3527,12 +3527,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>videoDuration</t>
+          <t>videoPlayCount</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>Duração do vídeo em segundos.</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -3554,12 +3554,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>videoDuration</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>double</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -3569,7 +3569,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
+          <t>Duração do vídeo em segundos.</t>
         </is>
       </c>
     </row>
@@ -3581,7 +3581,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -3596,7 +3596,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
+          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
         </is>
       </c>
     </row>
@@ -3608,7 +3608,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>shortCode</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -3623,7 +3623,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
+          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
         </is>
       </c>
     </row>
@@ -3635,12 +3635,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>isSponsored</t>
+          <t>shortCode</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Flag de conteúdo patrocinado no Reel (bruto do Apify).</t>
+          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
         </is>
       </c>
     </row>
@@ -3662,7 +3662,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>isCommentsDisabled</t>
+          <t>isSponsored</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -3677,7 +3677,7 @@
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Se os comentários estão desabilitados no post/reel.</t>
+          <t>Flag de conteúdo patrocinado no Reel (bruto do Apify).</t>
         </is>
       </c>
     </row>
@@ -3689,7 +3689,7 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>isPinned</t>
+          <t>isCommentsDisabled</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -3704,7 +3704,7 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Se o reel está fixado no perfil.</t>
+          <t>Se os comentários estão desabilitados no post/reel.</t>
         </is>
       </c>
     </row>
@@ -3716,12 +3716,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>latestComments</t>
+          <t>isPinned</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -3731,7 +3731,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Lista bruta (JSON) dos comentários mais recentes do reel ou post, retornada pelo Apify -- fonte de comments_clean (reels) e de post_comments_clean (posts de feed, issue #212).</t>
+          <t>Se o reel está fixado no perfil.</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3743,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>transcript</t>
+          <t>latestComments</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -3758,7 +3758,7 @@
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Transcrição de fala do reel, via flag paga includeTranscript do actor -- nullable (vídeo mudo/flag desligada).</t>
+          <t>Lista bruta (JSON) dos comentários mais recentes do reel ou post, retornada pelo Apify -- fonte de comments_clean (reels) e de post_comments_clean (posts de feed, issue #212).</t>
         </is>
       </c>
     </row>
@@ -3770,22 +3770,22 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>transcript</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Transcrição de fala do reel, via flag paga includeTranscript do actor -- nullable (vídeo mudo/flag desligada).</t>
         </is>
       </c>
     </row>
@@ -3797,12 +3797,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
@@ -3824,7 +3824,7 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>_source</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -3839,7 +3839,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
@@ -3851,7 +3851,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>_raw</t>
+          <t>_source</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -3866,19 +3866,19 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Bronze fiel (ADR 0039): o item COMPLETO retornado pela Apify, serializado como JSON string (ensure_ascii=False), inclusive campos que as colunas tipadas não modelam. Fonte para reprocessar a Silver sem nova extração; parsing e validação ficam na Silver. Substitui a antiga landing zone.</t>
+          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>ugc_mentions</t>
+          <t>instagram_reels</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>_raw</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -3888,12 +3888,12 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
+          <t>Bronze fiel (ADR 0039): o item COMPLETO retornado pela Apify, serializado como JSON string (ensure_ascii=False), inclusive campos que as colunas tipadas não modelam. Fonte para reprocessar a Silver sem nova extração; parsing e validação ficam na Silver. Substitui a antiga landing zone.</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>shortCode</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
+          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
         </is>
       </c>
     </row>
@@ -3932,7 +3932,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>shortCode</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -3947,7 +3947,7 @@
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
+          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
         </is>
       </c>
     </row>
@@ -3959,7 +3959,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>caption</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -3974,7 +3974,7 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Legenda/texto do post ou reel.</t>
+          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
         </is>
       </c>
     </row>
@@ -3986,7 +3986,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>mentions</t>
+          <t>caption</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -4001,7 +4001,7 @@
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Lista de usernames @-mencionados em legenda/comentário do post de UGC, serializada como JSON string -- só ~31% dos posts reais têm este campo preenchido.</t>
+          <t>Legenda/texto do post ou reel.</t>
         </is>
       </c>
     </row>
@@ -4013,7 +4013,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>taggedUsers</t>
+          <t>mentions</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -4028,7 +4028,7 @@
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Lista de objetos (um por pessoa marcada visualmente na foto/vídeo, com `username`/`full_name`/`is_verified`/`is_private`) do post de UGC, serializada como JSON string -- substitui o campo `matchTypes` (não existe no actor real); presente em ~69% dos posts, mais frequente que `mentions`.</t>
+          <t>Lista de usernames @-mencionados em legenda/comentário do post de UGC, serializada como JSON string -- só ~31% dos posts reais têm este campo preenchido.</t>
         </is>
       </c>
     </row>
@@ -4040,12 +4040,12 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>taggedUsers</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Lista de objetos (um por pessoa marcada visualmente na foto/vídeo, com `username`/`full_name`/`is_verified`/`is_private`) do post de UGC, serializada como JSON string -- substitui o campo `matchTypes` (não existe no actor real); presente em ~69% dos posts, mais frequente que `mentions`.</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>commentsCount</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -4082,7 +4082,7 @@
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Número de comentários.</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>videoPlayCount</t>
+          <t>commentsCount</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
+          <t>Número de comentários.</t>
         </is>
       </c>
     </row>
@@ -4121,12 +4121,12 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>videoPlayCount</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>ownerUsername</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Username de quem publicou o post de UGC (autor terceiro que marcou/mencionou o governador -- Bronze, nome real do actor apify/instagram-tagged-scraper). Normalizado para `authorUsername` na Silver.</t>
+          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
         </is>
       </c>
     </row>
@@ -4175,7 +4175,7 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>ownerFullName</t>
+          <t>ownerUsername</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -4190,7 +4190,7 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Nome completo de quem publicou o post de UGC (Bronze, confirmado pelo piloto real).</t>
+          <t>Username de quem publicou o post de UGC (autor terceiro que marcou/mencionou o governador -- Bronze, nome real do actor apify/instagram-tagged-scraper). Normalizado para `authorUsername` na Silver.</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>ownerId</t>
+          <t>ownerFullName</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>Id do perfil de quem publicou o post de UGC (autor terceiro, Bronze, confirmado pelo piloto real) -- distinto do `ownerId` de posts/reels, que é o próprio governador.</t>
+          <t>Nome completo de quem publicou o post de UGC (Bronze, confirmado pelo piloto real).</t>
         </is>
       </c>
     </row>
@@ -4229,12 +4229,12 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>paidPartnership</t>
+          <t>ownerId</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
@@ -4244,7 +4244,7 @@
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Flag de parceria paga (publi) declarada pelo Instagram no post de UGC -- único campo de publi que o actor real expõe (piloto 2026-09-19); `isAd`/`isAffiliate` da especificação original não existem.</t>
+          <t>Id do perfil de quem publicou o post de UGC (autor terceiro, Bronze, confirmado pelo piloto real) -- distinto do `ownerId` de posts/reels, que é o próprio governador.</t>
         </is>
       </c>
     </row>
@@ -4256,22 +4256,22 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>paidPartnership</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Flag de parceria paga (publi) declarada pelo Instagram no post de UGC -- único campo de publi que o actor real expõe (piloto 2026-09-19); `isAd`/`isAffiliate` da especificação original não existem.</t>
         </is>
       </c>
     </row>
@@ -4283,12 +4283,12 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -4298,7 +4298,7 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>_source</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
@@ -4337,27 +4337,54 @@
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
+          <t>_source</t>
+        </is>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>Origem do dado bruto -- sempre 'apify' hoje (src/data_extract/scraper.py).</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>ugc_mentions</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
           <t>_raw</t>
         </is>
       </c>
-      <c r="C77" s="3" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D77" s="3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E77" s="3" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>Bronze fiel (ADR 0039): o item COMPLETO retornado pela Apify, serializado como JSON string (ensure_ascii=False), inclusive campos que as colunas tipadas não modelam. Fonte para reprocessar a Silver sem nova extração; parsing e validação ficam na Silver. Substitui a antiga landing zone.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E77"/>
+  <autoFilter ref="A1:E78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4368,7 +4395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -5169,22 +5196,22 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>isPinned</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Se o reel está fixado no perfil.</t>
         </is>
       </c>
     </row>
@@ -5196,12 +5223,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -5211,7 +5238,7 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5250,7 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>_source_layer</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -5238,19 +5265,19 @@
       </c>
       <c r="E32" s="3" t="inlineStr">
         <is>
-          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>reels_clean</t>
+          <t>posts_clean</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>_source_layer</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -5265,7 +5292,7 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
+          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5304,7 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>ownerId</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -5292,7 +5319,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>Id do perfil (Bronze/Instagram) que publicou o post/reel.</t>
+          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
         </is>
       </c>
     </row>
@@ -5304,7 +5331,7 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>ownerUsername</t>
+          <t>ownerId</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -5319,7 +5346,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>Username do perfil que publicou o post/reel/comentário.</t>
+          <t>Id do perfil (Bronze/Instagram) que publicou o post/reel.</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5358,7 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>inputUrl</t>
+          <t>ownerUsername</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -5341,12 +5368,12 @@
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
+          <t>Username do perfil que publicou o post/reel/comentário.</t>
         </is>
       </c>
     </row>
@@ -5358,22 +5385,22 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>commentsCount</t>
+          <t>inputUrl</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>Número de comentários.</t>
+          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
         </is>
       </c>
     </row>
@@ -5385,7 +5412,7 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>commentsCount</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -5400,7 +5427,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Número de comentários.</t>
         </is>
       </c>
     </row>
@@ -5412,7 +5439,7 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>videoPlayCount</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -5422,12 +5449,12 @@
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -5439,12 +5466,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>videoDuration</t>
+          <t>videoPlayCount</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -5454,7 +5481,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>Duração do vídeo em segundos.</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -5466,22 +5493,22 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>data_hora</t>
+          <t>videoDuration</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us]</t>
+          <t>double</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>Timestamp parseado e convertido para America/Sao_Paulo (naive), a partir de `timestamp` bruto (PostCleaner._parse_timestamp).</t>
+          <t>Duração do vídeo em segundos.</t>
         </is>
       </c>
     </row>
@@ -5493,12 +5520,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>data_hora</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us]</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -5508,7 +5535,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>Granularidade fixada pelo cleaner: 'FEED' (posts_clean) ou 'REELS' (reels_clean) -- não confundir com `type_raw` (bruto do Apify).</t>
+          <t>Timestamp parseado e convertido para America/Sao_Paulo (naive), a partir de `timestamp` bruto (PostCleaner._parse_timestamp).</t>
         </is>
       </c>
     </row>
@@ -5520,7 +5547,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>type_raw</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -5530,12 +5557,12 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr">
         <is>
-          <t>Campo bruto `type` do Apify (Image/Video/Sidecar), preservado antes de `Tipo` (FEED/REELS) ser atribuído -- preditor de Formato da regressão de performance-por-post.</t>
+          <t>Granularidade fixada pelo cleaner: 'FEED' (posts_clean) ou 'REELS' (reels_clean) -- não confundir com `type_raw` (bruto do Apify).</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5574,7 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>shortCode</t>
+          <t>type_raw</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -5562,7 +5589,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
+          <t>Campo bruto `type` do Apify (Image/Video/Sidecar), preservado antes de `Tipo` (FEED/REELS) ser atribuído -- preditor de Formato da regressão de performance-por-post.</t>
         </is>
       </c>
     </row>
@@ -5574,12 +5601,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>isSponsored</t>
+          <t>shortCode</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -5589,7 +5616,7 @@
       </c>
       <c r="E45" s="3" t="inlineStr">
         <is>
-          <t>Flag de conteúdo patrocinado no Reel (bruto do Apify).</t>
+          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
         </is>
       </c>
     </row>
@@ -5601,7 +5628,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>isCommentsDisabled</t>
+          <t>isSponsored</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -5616,7 +5643,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>Se os comentários estão desabilitados no post/reel.</t>
+          <t>Flag de conteúdo patrocinado no Reel (bruto do Apify).</t>
         </is>
       </c>
     </row>
@@ -5628,22 +5655,22 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Total de Engajamento</t>
+          <t>isCommentsDisabled</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr">
         <is>
-          <t>likesCount + commentsCount deste reel (PostCleaner.clean_reels) -- por-REEL, insumo do PCA/AutoClusterHPO. Não confundir com 'TOTAL ENGAJAMENTO' (maiúsculo, com espaço) de governor_engagement, que é por-PERFIL agregado.</t>
+          <t>Se os comentários estão desabilitados no post/reel.</t>
         </is>
       </c>
     </row>
@@ -5655,12 +5682,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>transcript</t>
+          <t>isPinned</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -5670,7 +5697,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>Transcrição de fala do reel, via flag paga includeTranscript do actor -- nullable (vídeo mudo/flag desligada).</t>
+          <t>Se o reel está fixado no perfil.</t>
         </is>
       </c>
     </row>
@@ -5682,12 +5709,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>Total de Engajamento</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -5697,7 +5724,7 @@
       </c>
       <c r="E49" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>likesCount + commentsCount deste reel (PostCleaner.clean_reels) -- por-REEL, insumo do PCA/AutoClusterHPO. Não confundir com 'TOTAL ENGAJAMENTO' (maiúsculo, com espaço) de governor_engagement, que é por-PERFIL agregado.</t>
         </is>
       </c>
     </row>
@@ -5709,7 +5736,7 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>transcript</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -5719,12 +5746,12 @@
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Transcrição de fala do reel, via flag paga includeTranscript do actor -- nullable (vídeo mudo/flag desligada).</t>
         </is>
       </c>
     </row>
@@ -5736,12 +5763,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>_source_layer</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -5751,19 +5778,19 @@
       </c>
       <c r="E51" s="3" t="inlineStr">
         <is>
-          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>comments_clean</t>
+          <t>reels_clean</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>id_reel</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -5773,24 +5800,24 @@
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>Id da publicação (reel ou post) de origem do comentário/tópico -- chave de junção com reels_clean/posts_clean; em governor_sentiment, comentários de posts (origem_comentario == 'post') também usam esta coluna.</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>comments_clean</t>
+          <t>reels_clean</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>id_comment</t>
+          <t>_source_layer</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -5800,12 +5827,12 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Id único do comentário individual (pós-explosão de latestComments).</t>
+          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
@@ -5817,7 +5844,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id_reel</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -5832,7 +5859,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Texto avaliado -- comentário, legenda ou transcrição, dependendo da tabela/coluna `fonte`.</t>
+          <t>Id da publicação (reel ou post) de origem do comentário/tópico -- chave de junção com reels_clean/posts_clean; em governor_sentiment, comentários de posts (origem_comentario == 'post') também usam esta coluna.</t>
         </is>
       </c>
     </row>
@@ -5844,22 +5871,22 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>comprimento texto</t>
+          <t>id_comment</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr">
         <is>
-          <t>Número de caracteres de `text` -- usado para filtrar comentários &gt;= 512 caracteres (CommentCleaner.MAX_TEXT_LENGTH).</t>
+          <t>Id único do comentário individual (pós-explosão de latestComments).</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5898,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>ownerUsername</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -5886,7 +5913,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Username do perfil que publicou o post/reel/comentário.</t>
+          <t>Texto avaliado -- comentário, legenda ou transcrição, dependendo da tabela/coluna `fonte`.</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5925,7 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>comprimento texto</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -5908,12 +5935,12 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Número de caracteres de `text` -- usado para filtrar comentários &gt;= 512 caracteres (CommentCleaner.MAX_TEXT_LENGTH).</t>
         </is>
       </c>
     </row>
@@ -5925,12 +5952,12 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>repliesCount</t>
+          <t>ownerUsername</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
@@ -5940,7 +5967,7 @@
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>Número de respostas a um comentário.</t>
+          <t>Username do perfil que publicou o post/reel/comentário.</t>
         </is>
       </c>
     </row>
@@ -5952,12 +5979,12 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -5967,7 +5994,7 @@
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -5979,12 +6006,12 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>inputUrl</t>
+          <t>repliesCount</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -5994,7 +6021,7 @@
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
+          <t>Número de respostas a um comentário.</t>
         </is>
       </c>
     </row>
@@ -6006,22 +6033,22 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
         </is>
       </c>
     </row>
@@ -6033,7 +6060,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>inputUrl</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -6043,12 +6070,12 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
         </is>
       </c>
     </row>
@@ -6060,12 +6087,12 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>_source_layer</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
@@ -6075,19 +6102,19 @@
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>post_comments_clean</t>
+          <t>comments_clean</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>id_post</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -6097,24 +6124,24 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>Id do post de feed comentado (inclui reels capturados no grid de posts, issue #152) -- vira `id_reel` ao entrar em governor_sentiment.</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>post_comments_clean</t>
+          <t>comments_clean</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>id_comment</t>
+          <t>_source_layer</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -6124,12 +6151,12 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>Id único do comentário individual (pós-explosão de latestComments).</t>
+          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
@@ -6141,7 +6168,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>id_post</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -6156,7 +6183,7 @@
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>Texto avaliado -- comentário, legenda ou transcrição, dependendo da tabela/coluna `fonte`.</t>
+          <t>Id do post de feed comentado (inclui reels capturados no grid de posts, issue #152) -- vira `id_reel` ao entrar em governor_sentiment.</t>
         </is>
       </c>
     </row>
@@ -6168,22 +6195,22 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>comprimento texto</t>
+          <t>id_comment</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>Número de caracteres de `text` -- usado para filtrar comentários &gt;= 512 caracteres (CommentCleaner.MAX_TEXT_LENGTH).</t>
+          <t>Id único do comentário individual (pós-explosão de latestComments).</t>
         </is>
       </c>
     </row>
@@ -6195,7 +6222,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>ownerUsername</t>
+          <t>text</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -6210,7 +6237,7 @@
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>Username do perfil que publicou o post/reel/comentário.</t>
+          <t>Texto avaliado -- comentário, legenda ou transcrição, dependendo da tabela/coluna `fonte`.</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6249,7 @@
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>comprimento texto</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -6232,12 +6259,12 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E69" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Número de caracteres de `text` -- usado para filtrar comentários &gt;= 512 caracteres (CommentCleaner.MAX_TEXT_LENGTH).</t>
         </is>
       </c>
     </row>
@@ -6249,12 +6276,12 @@
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>repliesCount</t>
+          <t>ownerUsername</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
@@ -6264,7 +6291,7 @@
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>Número de respostas a um comentário.</t>
+          <t>Username do perfil que publicou o post/reel/comentário.</t>
         </is>
       </c>
     </row>
@@ -6276,12 +6303,12 @@
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>timestamp</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
@@ -6291,7 +6318,7 @@
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -6303,12 +6330,12 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>inputUrl</t>
+          <t>repliesCount</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
@@ -6318,7 +6345,7 @@
       </c>
       <c r="E72" s="3" t="inlineStr">
         <is>
-          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
+          <t>Número de respostas a um comentário.</t>
         </is>
       </c>
     </row>
@@ -6330,22 +6357,22 @@
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>timestamp</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E73" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Timestamp bruto do Apify, como string ISO -- ver `data_hora` para a versão já parseada/tipada (Silver).</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6384,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>inputUrl</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -6367,12 +6394,12 @@
       </c>
       <c r="D74" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E74" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
         </is>
       </c>
     </row>
@@ -6384,12 +6411,12 @@
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>_source_layer</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D75" s="3" t="inlineStr">
@@ -6399,19 +6426,19 @@
       </c>
       <c r="E75" s="3" t="inlineStr">
         <is>
-          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>governors_metadata</t>
+          <t>post_comments_clean</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>inputUrl</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -6426,19 +6453,19 @@
       </c>
       <c r="E76" s="3" t="inlineStr">
         <is>
-          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>governors_metadata</t>
+          <t>post_comments_clean</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>nome</t>
+          <t>_source_layer</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
@@ -6453,7 +6480,7 @@
       </c>
       <c r="E77" s="3" t="inlineStr">
         <is>
-          <t>Nome do governador (reference/governadores.xlsx, coluna 'Governador').</t>
+          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6492,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>uf</t>
+          <t>inputUrl</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -6475,12 +6502,12 @@
       </c>
       <c r="D78" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E78" s="3" t="inlineStr">
         <is>
-          <t>Unidade Federativa do governador (reference/governadores.xlsx, coluna 'Unidade Federativa').</t>
+          <t>URL do perfil de Instagram do governador (chave de junção mais usada entre perfis/posts/reels/Gold).</t>
         </is>
       </c>
     </row>
@@ -6492,7 +6519,7 @@
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>partido</t>
+          <t>nome</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -6502,12 +6529,12 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E79" s="3" t="inlineStr">
         <is>
-          <t>Partido do governador (reference/governadores.xlsx, coluna 'Partido').</t>
+          <t>Nome do governador (reference/governadores.xlsx, coluna 'Governador').</t>
         </is>
       </c>
     </row>
@@ -6519,22 +6546,22 @@
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>uf</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D80" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E80" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Unidade Federativa do governador (reference/governadores.xlsx, coluna 'Unidade Federativa').</t>
         </is>
       </c>
     </row>
@@ -6546,7 +6573,7 @@
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>partido</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -6556,12 +6583,12 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E81" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Partido do governador (reference/governadores.xlsx, coluna 'Partido').</t>
         </is>
       </c>
     </row>
@@ -6573,12 +6600,12 @@
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>_source_layer</t>
+          <t>_ingested_at</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us, tz=UTC]</t>
         </is>
       </c>
       <c r="D82" s="3" t="inlineStr">
@@ -6588,19 +6615,19 @@
       </c>
       <c r="E82" s="3" t="inlineStr">
         <is>
-          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>ugc_mentions</t>
+          <t>governors_metadata</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>id</t>
+          <t>_run_id</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -6610,24 +6637,24 @@
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E83" s="3" t="inlineStr">
         <is>
-          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>ugc_mentions</t>
+          <t>governors_metadata</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>shortCode</t>
+          <t>_source_layer</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -6637,12 +6664,12 @@
       </c>
       <c r="D84" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E84" s="3" t="inlineStr">
         <is>
-          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
+          <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
@@ -6654,7 +6681,7 @@
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>type</t>
+          <t>id</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -6669,7 +6696,7 @@
       </c>
       <c r="E85" s="3" t="inlineStr">
         <is>
-          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
+          <t>Identificador único do registro na origem (Instagram/Apify) -- semântica varia por tabela, ver coluna Grão.</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6708,7 @@
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>caption</t>
+          <t>shortCode</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -6696,7 +6723,7 @@
       </c>
       <c r="E86" s="3" t="inlineStr">
         <is>
-          <t>Legenda/texto do post ou reel.</t>
+          <t>Código curto do post/reel usado na URL pública do Instagram.</t>
         </is>
       </c>
     </row>
@@ -6708,7 +6735,7 @@
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>governor_username</t>
+          <t>type</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -6723,7 +6750,7 @@
       </c>
       <c r="E87" s="3" t="inlineStr">
         <is>
-          <t>Username do governador mencionado/marcado, resolvido cruzando `mentions` E `taggedUsers` (Bronze) com a lista de perfis conhecidos -- piloto real confirmou que ~69% dos posts só correlacionam via `taggedUsers`.</t>
+          <t>Tipo bruto do post retornado pelo Apify (Image/Video/Sidecar/Reel).</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6762,7 @@
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>authorUsername</t>
+          <t>caption</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -6750,7 +6777,7 @@
       </c>
       <c r="E88" s="3" t="inlineStr">
         <is>
-          <t>Username de quem publicou o post de UGC (autor, distinto do governador mencionado) -- campo normalizado na Silver; na Bronze o actor real só preenche `ownerUsername` (ver override específico de ugc_mentions, coluna `ownerUsername` colide de nome com posts/reels/comentários).</t>
+          <t>Legenda/texto do post ou reel.</t>
         </is>
       </c>
     </row>
@@ -6762,22 +6789,22 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>paidPartnership</t>
+          <t>governor_username</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>bool</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Flag de parceria paga (publi) declarada pelo Instagram no post de UGC -- único campo de publi que o actor real expõe (piloto 2026-09-19); `isAd`/`isAffiliate` da especificação original não existem.</t>
+          <t>Username do governador mencionado/marcado, resolvido cruzando `mentions` E `taggedUsers` (Bronze) com a lista de perfis conhecidos -- piloto real confirmou que ~69% dos posts só correlacionam via `taggedUsers`.</t>
         </is>
       </c>
     </row>
@@ -6789,22 +6816,22 @@
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>likesCount</t>
+          <t>authorUsername</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>string</t>
         </is>
       </c>
       <c r="D90" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E90" s="3" t="inlineStr">
         <is>
-          <t>Número de curtidas.</t>
+          <t>Username de quem publicou o post de UGC (autor, distinto do governador mencionado) -- campo normalizado na Silver; na Bronze o actor real só preenche `ownerUsername` (ver override específico de ugc_mentions, coluna `ownerUsername` colide de nome com posts/reels/comentários).</t>
         </is>
       </c>
     </row>
@@ -6816,12 +6843,12 @@
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>commentsCount</t>
+          <t>paidPartnership</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>bool</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
@@ -6831,7 +6858,7 @@
       </c>
       <c r="E91" s="3" t="inlineStr">
         <is>
-          <t>Número de comentários.</t>
+          <t>Flag de parceria paga (publi) declarada pelo Instagram no post de UGC -- único campo de publi que o actor real expõe (piloto 2026-09-19); `isAd`/`isAffiliate` da especificação original não existem.</t>
         </is>
       </c>
     </row>
@@ -6843,7 +6870,7 @@
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>videoPlayCount</t>
+          <t>likesCount</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
@@ -6853,12 +6880,12 @@
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
         <is>
-          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
+          <t>Número de curtidas.</t>
         </is>
       </c>
     </row>
@@ -6870,12 +6897,12 @@
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>data_hora</t>
+          <t>commentsCount</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us]</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
@@ -6885,7 +6912,7 @@
       </c>
       <c r="E93" s="3" t="inlineStr">
         <is>
-          <t>Timestamp parseado e convertido para America/Sao_Paulo (naive), a partir de `timestamp` bruto (PostCleaner._parse_timestamp).</t>
+          <t>Número de comentários.</t>
         </is>
       </c>
     </row>
@@ -6897,22 +6924,22 @@
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>_ingested_at</t>
+          <t>videoPlayCount</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
         <is>
-          <t>timestamp[us, tz=UTC]</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="D94" s="3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Sim</t>
         </is>
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+          <t>Reproduções (plays) do vídeo -- Reels/vídeo de feed. Nome correto da métrica: "reproduções (plays)", nunca "visualizações únicas" nem alcance. Insumo de Alcance/Profundidade do governor_scorecard e do estágio "Visualizações" do funil.</t>
         </is>
       </c>
     </row>
@@ -6924,12 +6951,12 @@
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>_run_id</t>
+          <t>data_hora</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
         <is>
-          <t>string</t>
+          <t>timestamp[us]</t>
         </is>
       </c>
       <c r="D95" s="3" t="inlineStr">
@@ -6939,7 +6966,7 @@
       </c>
       <c r="E95" s="3" t="inlineStr">
         <is>
-          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+          <t>Timestamp parseado e convertido para America/Sao_Paulo (naive), a partir de `timestamp` bruto (PostCleaner._parse_timestamp).</t>
         </is>
       </c>
     </row>
@@ -6951,27 +6978,81 @@
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
+          <t>_ingested_at</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>timestamp[us, tz=UTC]</t>
+        </is>
+      </c>
+      <c r="D96" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Timestamp UTC de quando o registro entrou na camada Bronze (BronzeWriter._add_ingestion_metadata).</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>ugc_mentions</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="inlineStr">
+        <is>
+          <t>_run_id</t>
+        </is>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Identificador da execução (src/run_id.py) que gravou a linha -- na Bronze, o run_id da Coleta (`coleta.py coletar`); como a Bronze é overwrite por Coleta, cada tabela Bronze tem um único run_id. Nas demais camadas, o da etapa que gravou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>ugc_mentions</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
           <t>_source_layer</t>
         </is>
       </c>
-      <c r="C96" s="3" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="D96" s="3" t="inlineStr">
-        <is>
-          <t>Não</t>
-        </is>
-      </c>
-      <c r="E96" s="3" t="inlineStr">
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="D98" s="3" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="E98" s="3" t="inlineStr">
         <is>
           <t>Camada de origem da linha na Silver -- 'bronze' para a maioria, 'raw_xlsx' só para governors_metadata.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E96"/>
+  <autoFilter ref="A1:E98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13181,7 +13262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -13189,9 +13270,10 @@
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="55" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13222,15 +13304,20 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
+          <t>Preço por resultado (verificado em 2026-10-13)</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
           <t>Parâmetros usados em produção</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Confiabilidade da fonte</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Notas</t>
         </is>
@@ -13264,15 +13351,20 @@
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
+          <t>Pay-per-event, evento 'result'. US$ por 1.000 resultados, por plano: Free 2,70 | Bronze 2,30 | Silver 1,90 | Gold 1,50 | Platinum 0,90 | Diamond 0,50.</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
           <t>directUrls=&lt;links&gt;, addParentData=False, resultsLimit=100, resultsType='details', searchType='user' (src/data_extract/scraper.py::InstagramScraper.scrape_profiles).</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>ID confirmado via api.apify.com/v2/acts/shu8hvrXbJbY3Eb9W -&gt; {"name":"instagram-scraper","username":"apify"} (docs/research/..., §0).</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>É o actor GENÉRICO "canivete suíço" da Apify, não o dedicado apify/instagram-profile-scraper -- rodado só em resultsType='details' hoje. O mesmo actor/ID também suporta resultsType='mentions'/'comments' e busca por hashtag, não explorado no pipeline atual (ver docs/research/..., §7.3, para a rota de UGC que reaproveitaria este mesmo actor sem integrar um novo).</t>
         </is>
@@ -13291,7 +13383,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>(resolvido pelo slug pela Apify -- não fixado como ID literal no código)</t>
+          <t>nH2AHrwxeTRJoN5hX (resolvido pelo slug pela Apify -- o código usa o slug, não o ID literal)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -13306,15 +13398,20 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
+          <t>Pay-per-event. Evento 'post', US$ por 1.000: Free 1,70 | Bronze 1,50 | Silver 1,30 | Gold 1,00 | Platinum 0,80 | Diamond 0,40. MAIS o evento 'post-details' ("post gravado com informação detalhada"), US$ por 1.000: Free 1,00 | Bronze 0,80 | Silver 0,70 | Gold 0,60 | Platinum 0,20 | Diamond 0,10. Se os dois incidem em cada post (a confirmar pelo faturamento da primeira Coleta de 90 dias), o total em Bronze é 2,30 por 1.000, igual aos demais actors. Add-on 'music-data' (Bronze 6,00 por 1.000 imagens/carrosséis com música) não usado.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
           <t>username=&lt;usernames&gt;, resultsLimit=30 (ScraperConfig.results_limit) + extra_run_input opcional (ex.: onlyPostsNewerThan, usado por src/coleta/coletar.py para o Recorte por janela relativa).</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>Confirmado via página do actor + input-schema (docs/research/..., §1.1) -- pay-per-event, ~$1.00/1.000 posts.</t>
-        </is>
-      </c>
       <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>Input-schema confirmado (docs/research/..., §1.1). Preço reverificado em 2026-10-13 pela API pública (api.apify.com/v2/acts/apify~instagram-post-scraper, pricingInfos mais recente); o '~$1.00/1.000' da pesquisa de 2026-09-08 está desatualizado (o preço mudou em 2026-03-10, 2026-07-13 e 2026-10-07).</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Não tem includeTranscript nem includeSharesCount (esses são do reel-scraper) -- não confundir com o actor genérico usado para perfis.</t>
         </is>
@@ -13333,7 +13430,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>(resolvido pelo slug pela Apify -- não fixado como ID literal no código)</t>
+          <t>xMc5Ga1oCONPmWJIa (resolvido pelo slug pela Apify -- o código usa o slug, não o ID literal)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -13348,15 +13445,20 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
+          <t>Pay-per-event. Evento 'reel', US$ por 1.000: Free 2,60 | Bronze 2,30 | Silver 1,40 | Gold 1,00 | Platinum 0,80 | Diamond 0,40. MAIS 'actor-start' de US$ 0,001 fixo por execução. Add-ons não habilitados hoje: 'shares-count' (Bronze 6,00 por 1.000 reels) e 'transcript' (Bronze US$ 0,041 por minuto iniciado de vídeo).</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
           <t>username=&lt;usernames&gt;, resultsLimit=30 + includeTranscript=True SOMENTE quando ScraperConfig.include_transcript=True (default False -- flag paga, cobrada por minuto de vídeo transcrito) + extra_run_input opcional.</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Confirmado via página do actor + input-schema (docs/research/..., §1.2) -- pay-per-event, ~$1.00/1.000 reels.</t>
-        </is>
-      </c>
       <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Input-schema confirmado (docs/research/..., §1.2). Preço reverificado em 2026-10-13 pela API pública (api.apify.com/v2/acts/apify~instagram-reel-scraper, pricingInfos mais recente); o '~$1.00/1.000' da pesquisa de 2026-09-08 não vale para o plano Bronze.</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Também suporta includeSharesCount (plano Starter+) e includeDownloadedVideo (cobrado por MB) -- nenhuma das duas está habilitada em ScraperConfig hoje (ver docs/research/..., §1.2, achado chave sobre sharesCount).</t>
         </is>
@@ -13375,7 +13477,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>(resolvido pelo slug pela Apify -- não fixado como ID literal no código)</t>
+          <t>zTSjdcGqjg6KEIBlt (resolvido pelo slug pela Apify -- o código usa o slug, não o ID literal)</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -13390,22 +13492,27 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
+          <t>Pay-per-event, evento 'post'. US$ por 1.000 posts, por plano: Free 2,70 | Bronze 2,30 | Silver 1,90 | Gold 1,50 | Platinum 1,00 | Diamond 0,50. A pesquisa de 2026-09-08 citava US$ 1,50 por 1.000, que hoje é o preço do plano Gold.</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
           <t>username=&lt;usernames&gt;, resultsLimit=&lt;baixo no piloto&gt; (ScraperConfig.mentions_actor_id, InstagramScraper.scrape_mentions).</t>
         </is>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>Escolhido sobre fetch_cat/instagram-mentions-scraper por reprodutibilidade (9.999 usuários, 5.0 estrelas vs. actor community "under maintenance", 2 usuários -- docs/research/..., §7.1). Schema de output confirmado 1:1 contra os 27 perfis do projeto pelo piloto real de 2026-09-19, e validado de novo pela execução de produção do mesmo dia.</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>docs/research/apify-instagram-actors-cobra-mapping.md (§7) também mapeia uma rota alternativa sem integrar actor novo: reconfigurar o actor de perfis já em uso (shu8hvrXbJbY3Eb9W) para resultsType='mentions' -- capacidade confirmada, schema de output dessa rota específica NÃO confirmado por exemplo primário.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5"/>
+  <autoFilter ref="A1:I5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>